<commit_message>
Add MV switchboards, pumps and MCCs; config 4 example
New equipment types: MV Busbar (switchboard with a breaker on every
way), Pump (MV motor load drawn as an M-circle) and MCC (box off an LV
board). Bus Coupler now also ties two MV busbars and prints its Notes
text (e.g. 'Normally open'). New bottom-up layout sizes each MV board
from its transformer/pump ways.

Config 4 example: two utility incomers onto two MV switchboards with a
normally-open tie, six riser feeders per board (3 transformers + 3
pumps), each transformer feeding an LV board with 2-3 MCCs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JnxbkkpjiEZhd9PqLAbPMc
</commit_message>
<xml_diff>
--- a/examples/config1_single_tx.xlsx
+++ b/examples/config1_single_tx.xlsx
@@ -1012,8 +1012,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown type" error="Pick one of: MV Incomer, RMU, Transformer, LV Busbar, Feeder, Bus Coupler" type="list">
-      <formula1>"MV Incomer,RMU,Transformer,LV Busbar,Feeder,Bus Coupler"</formula1>
+    <dataValidation sqref="B2:B60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown type" error="Pick one of: MV Incomer, MV Busbar, RMU, Transformer, Pump, LV Busbar, Feeder, MCC, Bus Coupler" type="list">
+      <formula1>"MV Incomer,MV Busbar,RMU,Transformer,Pump,LV Busbar,Feeder,MCC,Bus Coupler"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1026,7 +1026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1073,61 +1073,82 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Type: pick from the dropdown (MV Incomer, RMU, Transformer,</t>
+          <t xml:space="preserve">   - Type: pick from the dropdown (MV Incomer, MV Busbar, RMU,</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     LV Busbar, Feeder, Bus Coupler).</t>
+          <t xml:space="preserve">     Transformer, Pump, LV Busbar, Feeder, MCC, Bus Coupler).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Rating / Voltage: as read from the nameplate (e.g. 1000 kVA,</t>
+          <t xml:space="preserve">     MV Busbar = an MV switchboard; Pump = an MV motor load;</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     11/0.4 kV, 630 A, 400 V).</t>
+          <t xml:space="preserve">     MCC = motor control centre on an LV board. A Bus Coupler</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
+          <t xml:space="preserve">     between two MV Busbars is the bus tie.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+          <t xml:space="preserve">   - Rating / Voltage: as read from the nameplate (e.g. 1000 kVA,</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+          <t xml:space="preserve">     11/0.4 kV, 630 A, 400 V).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   and you get the single-line diagram as an SVG.</t>
         </is>

</xml_diff>

<commit_message>
Add Protection column: supply-side device per equipment row
New optional Protection column in the Equipment sheet and the
Sketchpad table: the device on the item's supply side - CB, LBS,
Fuse, Fuse-switch or Contactor (aliases accepted). Blank keeps the
default symbol, a comma list matches the Feeds From order, and free
text on a busbar (e.g. '87B differential') prints as a label
annotation. Protection never affects topology - only Feeds From does.

Both renderers draw the chosen symbol on the connection: RMU way
overrides, MV switchboard ways, LV incomers (split case per panel),
feeders and MCCs. Warnings for protection on an MV incomer (utility
side) and for unrecognised values. Example workbooks and presets now
carry full protection data; drawings are unchanged where the data
matches the old defaults.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JnxbkkpjiEZhd9PqLAbPMc
</commit_message>
<xml_diff>
--- a/examples/config1_single_tx.xlsx
+++ b/examples/config1_single_tx.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -520,8 +520,9 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -552,10 +553,15 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
           <t>Feeds From</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -584,7 +590,8 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Cable from utility</t>
         </is>
@@ -618,10 +625,15 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>LBS</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>MV1</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -651,10 +663,15 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>Fuse-switch</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>RMU1</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -684,10 +701,15 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>TX1</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -717,10 +739,15 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>BB1</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -750,10 +777,15 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>BB1</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -783,10 +815,15 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
           <t>BB1</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -816,10 +853,15 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>BB1</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -829,6 +871,7 @@
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -838,6 +881,7 @@
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -847,6 +891,7 @@
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -856,6 +901,7 @@
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -865,6 +911,7 @@
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -874,6 +921,7 @@
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -883,6 +931,7 @@
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -892,6 +941,7 @@
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -901,6 +951,7 @@
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -910,6 +961,7 @@
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -919,6 +971,7 @@
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -928,6 +981,7 @@
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -937,6 +991,7 @@
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -946,6 +1001,7 @@
       <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -955,6 +1011,7 @@
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -964,6 +1021,7 @@
       <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -973,6 +1031,7 @@
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -982,6 +1041,7 @@
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -991,6 +1051,7 @@
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -1000,6 +1061,7 @@
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -1009,11 +1071,15 @@
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown type" error="Pick one of: MV Incomer, MV Busbar, RMU, Transformer, Pump, LV Busbar, Feeder, MCC, Bus Coupler" type="list">
       <formula1>"MV Incomer,MV Busbar,RMU,Transformer,Pump,LV Busbar,Feeder,MCC,Bus Coupler"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CB,LBS,Fuse,Fuse-switch,Contactor"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1026,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1122,33 +1188,68 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
+          <t xml:space="preserve">   - Protection: the device on THIS item's supply side - pick</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+          <t xml:space="preserve">     CB, LBS, Fuse, Fuse-switch or Contactor, or leave blank for</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+          <t xml:space="preserve">     the usual default. Two supplies: comma list in the same</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+          <t xml:space="preserve">     order as Feeds From (e.g. LBS, CB). Free text on a busbar</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     (e.g. 87B differential) is printed next to its label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   and you get the single-line diagram as an SVG.</t>
         </is>

</xml_diff>

<commit_message>
Revise symbols per IEC 60617: breaker blade+X, add Fuse-contactor
- Circuit breaker is now the full IEC symbol: a switch blade with the
  X at its contact point (the bare X on the line was a shorthand).
  Applies to every breaker including bus couplers/ties, which now
  draw their actual device kind.
- New Fuse-contactor protection kind (aliases: fused contactor,
  contactor-fuse, motor starter) - back-up fuse in series with the
  contactor, the usual MV motor starter. Config 4 pumps use it.
- Legend gains the fused contactor cell (12 items, tighter cells).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JnxbkkpjiEZhd9PqLAbPMc
</commit_message>
<xml_diff>
--- a/examples/config1_single_tx.xlsx
+++ b/examples/config1_single_tx.xlsx
@@ -1079,7 +1079,7 @@
       <formula1>"MV Incomer,MV Busbar,RMU,Transformer,Pump,LV Busbar,Feeder,MCC,Bus Coupler"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"CB,LBS,Fuse,Fuse-switch,Contactor"</formula1>
+      <formula1>"CB,LBS,Fuse,Fuse-switch,Contactor,Fuse-contactor"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1195,61 +1195,68 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     CB, LBS, Fuse, Fuse-switch or Contactor, or leave blank for</t>
+          <t xml:space="preserve">     CB, LBS, Fuse, Fuse-switch, Contactor or Fuse-contactor (an</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     the usual default. Two supplies: comma list in the same</t>
+          <t xml:space="preserve">     MV motor starter = fuse + contactor), or leave blank for</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     order as Feeds From (e.g. LBS, CB). Free text on a busbar</t>
+          <t xml:space="preserve">     the usual default. Two supplies: comma list in the same</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     (e.g. 87B differential) is printed next to its label.</t>
+          <t xml:space="preserve">     order as Feeds From (e.g. LBS, CB). Free text on a busbar</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
+          <t xml:space="preserve">     (e.g. 87B differential) is printed next to its label.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   and you get the single-line diagram as an SVG.</t>
         </is>

</xml_diff>

<commit_message>
Add SU Transformer type: a step-up drawn under its MV board
A step-up could only be drawn above the board (fixed Y_GEN/Y_SU_C1
constants with headroom added on top), so generation that belongs
below the board had no way to be sketched.

New 'SU Transformer' type (aliases su tx, step-up transformer, step
up) draws the same column rotated 180 degrees: it occupies a way of
the board like a step-down - Feeds From is that board - dropping
through its Protection device to the transformer, with the
generation source hanging below it (the generator's Feeds From is
the SU Transformer). A plain Transformer feeding an MV board keeps
the above-the-board column.

Both renderers, plus the workbook dropdown and how-to text. Existing
drawings unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JnxbkkpjiEZhd9PqLAbPMc
</commit_message>
<xml_diff>
--- a/examples/config1_single_tx.xlsx
+++ b/examples/config1_single_tx.xlsx
@@ -1075,8 +1075,8 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown type" error="Pick one of: MV Incomer, Generator, MV Busbar, RMU, Transformer, Pump, LV Busbar, Feeder, MCC, Bus Coupler" type="list">
-      <formula1>"MV Incomer,Generator,MV Busbar,RMU,Transformer,Pump,LV Busbar,Feeder,MCC,Bus Coupler"</formula1>
+    <dataValidation sqref="B2:B60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown type" error="Pick one of: MV Incomer, Generator, MV Busbar, RMU, Transformer, SU Transformer, Pump, LV Busbar, Feeder, MCC, Bus Coupler" type="list">
+      <formula1>"MV Incomer,Generator,MV Busbar,RMU,Transformer,SU Transformer,Pump,LV Busbar,Feeder,MCC,Bus Coupler"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"CB,LBS,Fuse,Fuse-switch,Contactor,Fuse-contactor"</formula1>
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1146,124 +1146,152 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Busbar, RMU, Transformer, Pump, LV Busbar, Feeder, MCC,</t>
+          <t xml:space="preserve">     Busbar, RMU, Transformer, SU Transformer, Pump, LV Busbar,</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Bus Coupler).</t>
+          <t xml:space="preserve">     Feeder, MCC, Bus Coupler).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     MV Busbar = an MV switchboard; Pump = an MV motor load;</t>
+          <t xml:space="preserve">     SU Transformer = a step-up drawn hanging UNDER its MV board</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     MCC = motor control centre on an LV board. A Bus Coupler</t>
+          <t xml:space="preserve">     (Feeds From = that board), with its generator below it</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     between two MV Busbars is the bus tie.</t>
+          <t xml:space="preserve">     (the generator's Feeds From = the SU Transformer). A plain</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Rating / Voltage: as read from the nameplate (e.g. 1000 kVA,</t>
+          <t xml:space="preserve">     Transformer that feeds an MV board is drawn above it.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     11/0.4 kV, 630 A, 400 V).</t>
+          <t xml:space="preserve">     MV Busbar = an MV switchboard; Pump = an MV motor load;</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Protection: the device on THIS item's supply side - pick</t>
+          <t xml:space="preserve">     MCC = motor control centre on an LV board. A Bus Coupler</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     CB, LBS, Fuse, Fuse-switch, Contactor or Fuse-contactor (an</t>
+          <t xml:space="preserve">     between two MV Busbars is the bus tie.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     MV motor starter = fuse + contactor), or leave blank for</t>
+          <t xml:space="preserve">   - Rating / Voltage: as read from the nameplate (e.g. 1000 kVA,</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     the usual default. Two supplies: comma list in the same</t>
+          <t xml:space="preserve">     11/0.4 kV, 630 A, 400 V).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     order as Feeds From (e.g. LBS, CB). Free text on a busbar</t>
+          <t xml:space="preserve">   - Protection: the device on THIS item's supply side - pick</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     (e.g. 87B differential) is printed next to its label.</t>
+          <t xml:space="preserve">     CB, LBS, Fuse, Fuse-switch, Contactor or Fuse-contactor (an</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
+          <t xml:space="preserve">     MV motor starter = fuse + contactor), or leave blank for</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+          <t xml:space="preserve">     the usual default. Two supplies: comma list in the same</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+          <t xml:space="preserve">     order as Feeds From (e.g. LBS, CB). Free text on a busbar</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+          <t xml:space="preserve">     (e.g. 87B differential) is printed next to its label.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   and you get the single-line diagram as an SVG.</t>
         </is>

</xml_diff>

<commit_message>
Motors and feeders under an MCC
An MCC with loads becomes a little board of its own on the row below:
the box stays on the board's feeder band, a bus hangs under it and the
motors and feeders take their ways off that bus, a contactor as the
default starter. Both engines; the checker lets an MCC own its bus.
New feature sheet tests/features/f6_mcc.xlsx.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JnxbkkpjiEZhd9PqLAbPMc
</commit_message>
<xml_diff>
--- a/examples/config1_single_tx.xlsx
+++ b/examples/config1_single_tx.xlsx
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1209,166 +1209,173 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     MCC = motor control centre on an LV board. A Bus Coupler</t>
+          <t xml:space="preserve">     MCC = motor control centre on an LV board; a Pump or Feeder</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     between two MV Busbars is the bus tie; one between a board</t>
+          <t xml:space="preserve">     can feed from an MCC and hangs off its own bus. A Bus Coupler</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     and a Generator is a changeover (ATS). A Generator can also</t>
+          <t xml:space="preserve">     between two MV Busbars is the bus tie; one between a board</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     feed a board directly: name it in the board's Feeds From.</t>
+          <t xml:space="preserve">     and a Generator is a changeover (ATS). A Generator can also</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     An LV Busbar fed from a Feeder or another LV Busbar is a</t>
+          <t xml:space="preserve">     feed a board directly: name it in the board's Feeds From.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     sub-board, drawn on the row below. A Feeder on MV gear is</t>
+          <t xml:space="preserve">     An LV Busbar fed from a Feeder or another LV Busbar is a</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     an outgoing cable way. Capacitor Bank, Earthing/NER and</t>
+          <t xml:space="preserve">     sub-board, drawn on the row below. A Feeder on MV gear is</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Surge Arrester need no load; a Feeder whose words say</t>
+          <t xml:space="preserve">     an outgoing cable way. Capacitor Bank, Earthing/NER and</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     capacitor / NER / arrester is drawn as one anyway.</t>
+          <t xml:space="preserve">     Surge Arrester need no load; a Feeder whose words say</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Notes: 'VSD' on a motor draws a drive box, 'Spare' dashes</t>
+          <t xml:space="preserve">     capacitor / NER / arrester is drawn as one anyway.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     the way, 'N.O.' on an RMU marks the ring's open point.</t>
+          <t xml:space="preserve">     Notes: 'VSD' on a motor draws a drive box, 'Spare' dashes</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Rating / Voltage: as read from the nameplate (e.g. 1000 kVA,</t>
+          <t xml:space="preserve">     the way, 'N.O.' on an RMU marks the ring's open point.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     11/0.4 kV, 630 A, 400 V).</t>
+          <t xml:space="preserve">   - Rating / Voltage: as read from the nameplate (e.g. 1000 kVA,</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Protection: the device on THIS item's supply side - pick</t>
+          <t xml:space="preserve">     11/0.4 kV, 630 A, 400 V).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     CB, LBS, Fuse, Fuse-switch, Contactor or Fuse-contactor (an</t>
+          <t xml:space="preserve">   - Protection: the device on THIS item's supply side - pick</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     MV motor starter = fuse + contactor), or leave blank for</t>
+          <t xml:space="preserve">     CB, LBS, Fuse, Fuse-switch, Contactor or Fuse-contactor (an</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     the usual default. Two supplies: comma list in the same</t>
+          <t xml:space="preserve">     MV motor starter = fuse + contactor), or leave blank for</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     order as Feeds From (e.g. LBS, CB). Free text on a busbar</t>
+          <t xml:space="preserve">     the usual default. Two supplies: comma list in the same</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     (e.g. 87B differential) is printed next to its label.</t>
+          <t xml:space="preserve">     order as Feeds From (e.g. LBS, CB). Free text on a busbar</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
+          <t xml:space="preserve">     (e.g. 87B differential) is printed next to its label.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   and you get the single-line diagram as an SVG.</t>
         </is>

</xml_diff>

<commit_message>
A how-to-fill page in the Sketchpad and a fuller one in the workbook
Every column, every type and how it draws, the wiring recipes, and the
words in Description / Notes that change a symbol (VSD, Spare, N.O.,
capacitor, NER, arrester), so a surveyor can find out that a drive is
drawn by writing VSD without reading the README. Opened from a header
button or the link under the table; the same text on the workbook's
How to fill sheet.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JnxbkkpjiEZhd9PqLAbPMc
</commit_message>
<xml_diff>
--- a/examples/config1_single_tx.xlsx
+++ b/examples/config1_single_tx.xlsx
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1118,266 +1118,617 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>1. Info sheet: site name, date, surveyor, free notes.</t>
+          <t>One row per item, top of the network first. The drawing's topology</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2. Equipment sheet: one row per item, top of the network first.</t>
+          <t>comes only from ID and Feeds From: an item is drawn under whatever it</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - ID: short unique tag you invent (MV1, RMU1, TX1, BB1, F1...).</t>
+          <t>feeds from. Row order sets left-to-right order. A half-filled row still</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Type: pick from the dropdown (MV Incomer, Generator, MV</t>
+          <t>draws, with an open terminal where the supply or the load is missing.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Busbar, RMU, Transformer, Pump, LV Busbar, Feeder, MCC,</t>
-        </is>
-      </c>
+      <c r="A8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Bus Coupler, Capacitor Bank, Earthing/NER, Surge Arrester).</t>
+          <t>COLUMNS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     One Transformer type covers step-down and step-up: which</t>
+          <t xml:space="preserve">  ID          a short unique tag you invent: MV1, RMU1, TX1, BB1, F1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     way it is drawn follows Feeds From. A transformer that</t>
+          <t xml:space="preserve">  Type        pick from the dropdown (see TYPES)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     feeds an MV board is a step-up, drawn above it with its</t>
+          <t xml:space="preserve">  Description free text, printed as a label (a few words also change</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     source on top; one hung under an MV board whose load is a</t>
+          <t xml:space="preserve">              the symbol - see WORDS)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Generator is the same step-up drawn upside down. Write</t>
+          <t xml:space="preserve">  Rating      from the nameplate: 1000 kVA, 630 A, 315 kW</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     'step-up' in Description - the voltages say it too.</t>
+          <t xml:space="preserve">  Voltage     from the nameplate: 11/0.4 kV, 400 V - printed only</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     MV Busbar = an MV switchboard; Pump = an MV motor load;</t>
+          <t xml:space="preserve">  Protection  the device on THIS item's supply side: CB, LBS, Fuse,</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     MCC = motor control centre on an LV board; a Pump or Feeder</t>
+          <t xml:space="preserve">              Fuse-switch, Contactor, Fuse-contactor; blank = the usual</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     can feed from an MCC and hangs off its own bus. A Bus Coupler</t>
+          <t xml:space="preserve">              default; two supplies: a comma list in Feeds From order</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     between two MV Busbars is the bus tie; one between a board</t>
+          <t xml:space="preserve">              (LBS, CB). Free text on a busbar (87B differential) is</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     and a Generator is a changeover (ATS). A Generator can also</t>
+          <t xml:space="preserve">              printed as a zone label.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     feed a board directly: name it in the board's Feeds From.</t>
+          <t xml:space="preserve">  Feeds From  the ID of the item supplying this one; comma for two</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     An LV Busbar fed from a Feeder or another LV Busbar is a</t>
+          <t xml:space="preserve">              supplies (BB1, BB2 - MV1, MV2)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     sub-board, drawn on the row below. A Feeder on MV gear is</t>
+          <t xml:space="preserve">  Notes       anything worth remembering; printed on ties; a few</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     an outgoing cable way. Capacitor Bank, Earthing/NER and</t>
+          <t xml:space="preserve">              leading words change the symbol - see WORDS</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Surge Arrester need no load; a Feeder whose words say</t>
-        </is>
-      </c>
+      <c r="A25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     capacitor / NER / arrester is drawn as one anyway.</t>
+          <t>TYPES (and how each one draws)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Notes: 'VSD' on a motor draws a drive box, 'Spare' dashes</t>
+          <t xml:space="preserve">  MV Incomer     source tick at the top; feeds an MV Busbar, RMU or TX</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     the way, 'N.O.' on an RMU marks the ring's open point.</t>
+          <t xml:space="preserve">  MV Busbar      thick bar, a breaker on every way; a board fed from</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Rating / Voltage: as read from the nameplate (e.g. 1000 kVA,</t>
+          <t xml:space="preserve">                 another board sits one tier lower</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     11/0.4 kV, 630 A, 400 V).</t>
+          <t xml:space="preserve">  RMU            dashed enclosure, load-break switches on the ways in,</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Protection: the device on THIS item's supply side - pick</t>
+          <t xml:space="preserve">                 fuse-switches on the tee-offs; RMUs that feed from</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     CB, LBS, Fuse, Fuse-switch, Contactor or Fuse-contactor (an</t>
+          <t xml:space="preserve">                 each other form a ring side by side</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     MV motor starter = fuse + contactor), or leave blank for</t>
+          <t xml:space="preserve">  Transformer    two circles; step-down or step-up follows Feeds From</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     the usual default. Two supplies: comma list in the same</t>
+          <t xml:space="preserve">  Generator      G circle over the board it feeds, on top of a step-up</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     order as Feeds From (e.g. LBS, CB). Free text on a busbar</t>
+          <t xml:space="preserve">                 column, or under a reversed one</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     (e.g. 87B differential) is printed next to its label.</t>
+          <t xml:space="preserve">  Pump           M 3~ circle: transformer row on MV gear, feeder band</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Feeds From: the ID of the item supplying this one. Use a comma</t>
+          <t xml:space="preserve">                 on an LV board or an MCC, under a transformer of its own</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     for two supplies (bus coupler between BB1, BB2 - or an RMU fed</t>
+          <t xml:space="preserve">  LV Busbar      thick bar with its feeders; fed from a Feeder or</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">     by ring incomers MV1, MV2).</t>
+          <t xml:space="preserve">                 another LV Busbar it is a sub-board on the row below</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>3. Back at the office:  python sld_sketch.py thisfile.xlsx</t>
+          <t xml:space="preserve">  Feeder         drop + device + arrow; on MV gear an outgoing cable</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   and you get the single-line diagram as an SVG.</t>
+          <t xml:space="preserve">  MCC            labelled box; with Pumps/Feeders under it, a bus of</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 its own on the row below with the motor ways off it</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bus Coupler    breaker between two busbars of the same kind; between</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 a board and a Generator, a changeover (ATS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Capacitor Bank plates to earth (LV board or MV gear); needs no load</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Earthing/NER   resistor box to earth; needs no load</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Surge Arrester arrester box to earth; needs no load</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>WIRING RECIPES (Feeds From)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Step-down: TX feeds from the MV board/RMU; the LV Busbar from TX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Step-up from a genset or PV board: TX feeds from the Generator (or</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    generation LV Busbar); the MV Busbar/RMU feeds from TX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Step-up from a live LV board: TX feeds from that board; the MV</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    gear feeds from TX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Genset straight onto a board: the board feeds from MV, DG1, DG2;</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    the Generator rows have Feeds From blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Standby set on a changeover: a Bus Coupler row ATS feeding from</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    MSB3, G1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sub-board (DB): the LV Busbar feeds from the Feeder that supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    it, or straight from the main LV Busbar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Motors in an MCC: the MCC feeds from the board; each Pump from the MCC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bus tie: a Bus Coupler feeding from BB1, BB2; Notes Normally open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Board with two supplies: the board feeds from TX1, TX2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ring of RMUs from a board: each RMU feeds from its neighbours</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (PB, R2 ... R4, PB); a link written on both rows is drawn once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Open point of a ring: Notes on one RMU: N.O. towards RMU2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Spur or sub-ring off an RMU: the spur RMU feeds from the ring RMU;</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    a sub-ring's two RMUs feed from it and from each other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Several voltage levels: the lower board feeds from the transformer,</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    the transformer from the upper board; tiers follow the wiring,</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    never the Voltage column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Outgoing MV cable, capacitor bank, NER: a Feeder, Capacitor Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    or Earthing/NER row feeding from the MV board or RMU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>WORDS THAT CHANGE THE SYMBOL (read from Description and Notes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  VSD / VFD / drive        on a Pump: a drive box on the motor's drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Spare / Future /         at the start of Notes: the way drawn dashed</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Out of service</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  N.O. / Normally open     on a Bus Coupler: printed under it</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  N.O. towards RMU2,       on an RMU: an N.O. marker on the cable to</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ring open here           the RMU named, or under the box</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  capacitor / PFC / kvar   on a Feeder: drawn as a capacitor bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NER / earthing / zig-zag on a Feeder, or a Transformer with nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                           on its output: earthing resistor / tx</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  arrester / surge         on a Feeder: drawn as a surge arrester</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Protection words: CB MCCB MCB ACB - LBS isolator - Fuse -</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Fuse-switch SFU - Contactor - Fuse-contactor starter</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>BACK AT THE OFFICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  python sld_sketch.py thisfile.xlsx           -&gt; the SVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  python sld_sketch.py thisfile.xlsx --dxf     -&gt; SVG + DXF with the</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                  equipment table</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  python sld_check.py thisfile.xlsx            -&gt; checks the drawing</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                  against the table</t>
         </is>
       </c>
     </row>

</xml_diff>